<commit_message>
Roolit excelmuutos - jotta uusi raportti näkyy
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markusva/repos/Github/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395E9FDC-2890-D84A-A4EF-17F619C2C236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57BA7F91-4BAF-F64C-8854-7A35EA535044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40160" yWindow="-5300" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2065" uniqueCount="293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2078" uniqueCount="294">
   <si>
     <t xml:space="preserve">Roolimääritysten selitykset: </t>
   </si>
@@ -945,6 +945,9 @@
   </si>
   <si>
     <t>Välikatselmus</t>
+  </si>
+  <si>
+    <t>Vastaanottotarkastusraportti - MHU</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1219,6 +1222,21 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1555,7 +1573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Y144"/>
+  <dimension ref="A1:Y145"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.5" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -7592,85 +7610,65 @@
       <c r="X104" s="21"/>
       <c r="Y104" s="12"/>
     </row>
-    <row r="105" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A105" s="20" t="s">
+    <row r="105" spans="1:25" x14ac:dyDescent="0.15">
+      <c r="A105" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="B105" s="20" t="s">
-        <v>208</v>
-      </c>
-      <c r="C105" s="21"/>
-      <c r="D105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="E105" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="F105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="G105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="H105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="I105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="J105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="K105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L105" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="N105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O105" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P105" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q105" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="R105" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="S105" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="T105" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U105" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="V105" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="W105" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="X105" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y105" s="12"/>
+      <c r="B105" s="46" t="s">
+        <v>293</v>
+      </c>
+      <c r="C105" s="47"/>
+      <c r="D105" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="E105" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="F105" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="G105" s="47"/>
+      <c r="H105" s="47"/>
+      <c r="I105" s="47"/>
+      <c r="J105" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="K105" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="L105" s="49" t="s">
+        <v>38</v>
+      </c>
+      <c r="M105" s="47"/>
+      <c r="N105" s="48" t="s">
+        <v>38</v>
+      </c>
+      <c r="O105" s="47"/>
+      <c r="P105" s="47"/>
+      <c r="Q105" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="R105" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="S105" s="48" t="s">
+        <v>39</v>
+      </c>
+      <c r="T105" s="47"/>
+      <c r="U105" s="47"/>
+      <c r="V105" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="W105" s="47"/>
+      <c r="X105" s="47"/>
+      <c r="Y105" s="50"/>
     </row>
     <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="20" t="s">
         <v>168</v>
       </c>
       <c r="B106" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C106" s="21"/>
       <c r="D106" s="22" t="s">
@@ -7743,7 +7741,7 @@
         <v>168</v>
       </c>
       <c r="B107" s="20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C107" s="21"/>
       <c r="D107" s="22" t="s">
@@ -7816,7 +7814,7 @@
         <v>168</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C108" s="21"/>
       <c r="D108" s="22" t="s">
@@ -7835,10 +7833,10 @@
         <v>38</v>
       </c>
       <c r="I108" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J108" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K108" s="22" t="s">
         <v>38</v>
@@ -7847,7 +7845,7 @@
         <v>38</v>
       </c>
       <c r="M108" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N108" s="22" t="s">
         <v>38</v>
@@ -7876,7 +7874,9 @@
       <c r="V108" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="W108" s="21"/>
+      <c r="W108" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="X108" s="22" t="s">
         <v>39</v>
       </c>
@@ -7887,115 +7887,115 @@
         <v>168</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C109" s="21"/>
       <c r="D109" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="E109" s="25"/>
-      <c r="F109" s="21"/>
-      <c r="G109" s="21"/>
-      <c r="H109" s="21"/>
-      <c r="I109" s="21"/>
-      <c r="J109" s="21"/>
-      <c r="K109" s="21"/>
-      <c r="L109" s="25"/>
-      <c r="M109" s="21"/>
-      <c r="N109" s="21"/>
-      <c r="O109" s="21"/>
-      <c r="P109" s="21"/>
-      <c r="Q109" s="21"/>
-      <c r="R109" s="21"/>
-      <c r="S109" s="21"/>
-      <c r="T109" s="21"/>
-      <c r="U109" s="21"/>
-      <c r="V109" s="21"/>
+      <c r="E109" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F109" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="G109" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="H109" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="I109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="J109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="K109" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L109" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N109" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O109" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="R109" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="S109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="T109" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U109" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="V109" s="22" t="s">
+        <v>44</v>
+      </c>
       <c r="W109" s="21"/>
-      <c r="X109" s="21"/>
+      <c r="X109" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="Y109" s="12"/>
     </row>
     <row r="110" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A110" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="B110" s="39" t="s">
-        <v>285</v>
+      <c r="B110" s="20" t="s">
+        <v>212</v>
       </c>
       <c r="C110" s="21"/>
       <c r="D110" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="E110" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="F110" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="G110" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="H110" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="I110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="J110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="K110" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L110" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="N110" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O110" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="R110" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="S110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="T110" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U110" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="V110" s="22" t="s">
-        <v>44</v>
-      </c>
+      <c r="E110" s="25"/>
+      <c r="F110" s="21"/>
+      <c r="G110" s="21"/>
+      <c r="H110" s="21"/>
+      <c r="I110" s="21"/>
+      <c r="J110" s="21"/>
+      <c r="K110" s="21"/>
+      <c r="L110" s="25"/>
+      <c r="M110" s="21"/>
+      <c r="N110" s="21"/>
+      <c r="O110" s="21"/>
+      <c r="P110" s="21"/>
+      <c r="Q110" s="21"/>
+      <c r="R110" s="21"/>
+      <c r="S110" s="21"/>
+      <c r="T110" s="21"/>
+      <c r="U110" s="21"/>
+      <c r="V110" s="21"/>
       <c r="W110" s="21"/>
-      <c r="X110" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="X110" s="21"/>
       <c r="Y110" s="12"/>
     </row>
-    <row r="111" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A111" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="B111" s="20" t="s">
-        <v>213</v>
+      <c r="B111" s="39" t="s">
+        <v>285</v>
       </c>
       <c r="C111" s="21"/>
       <c r="D111" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E111" s="23" t="s">
         <v>38</v>
@@ -8016,7 +8016,7 @@
         <v>39</v>
       </c>
       <c r="K111" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L111" s="23" t="s">
         <v>38</v>
@@ -8037,34 +8037,32 @@
         <v>39</v>
       </c>
       <c r="R111" s="22" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S111" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="T111" s="22" t="s">
         <v>44</v>
       </c>
       <c r="U111" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V111" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="W111" s="22" t="s">
-        <v>40</v>
-      </c>
+      <c r="W111" s="21"/>
       <c r="X111" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Y111" s="12"/>
     </row>
-    <row r="112" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A112" s="20" t="s">
         <v>168</v>
       </c>
       <c r="B112" s="20" t="s">
-        <v>167</v>
+        <v>213</v>
       </c>
       <c r="C112" s="21"/>
       <c r="D112" s="22" t="s">
@@ -8089,7 +8087,7 @@
         <v>39</v>
       </c>
       <c r="K112" s="22" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L112" s="23" t="s">
         <v>38</v>
@@ -8110,25 +8108,25 @@
         <v>39</v>
       </c>
       <c r="R112" s="22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S112" s="22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="T112" s="22" t="s">
         <v>44</v>
       </c>
       <c r="U112" s="22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="V112" s="22" t="s">
         <v>44</v>
       </c>
       <c r="W112" s="22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="X112" s="22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="Y112" s="12"/>
     </row>
@@ -8137,29 +8135,35 @@
         <v>168</v>
       </c>
       <c r="B113" s="20" t="s">
-        <v>214</v>
+        <v>167</v>
       </c>
       <c r="C113" s="21"/>
       <c r="D113" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E113" s="23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="F113" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="G113" s="21"/>
-      <c r="H113" s="21"/>
-      <c r="I113" s="21"/>
+      <c r="G113" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="H113" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="I113" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="J113" s="22" t="s">
         <v>39</v>
       </c>
       <c r="K113" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L113" s="23" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="M113" s="22" t="s">
         <v>39</v>
@@ -8167,41 +8171,51 @@
       <c r="N113" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="O113" s="21"/>
-      <c r="P113" s="21"/>
+      <c r="O113" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P113" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="Q113" s="22" t="s">
         <v>39</v>
       </c>
       <c r="R113" s="22" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="S113" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="T113" s="21"/>
+        <v>39</v>
+      </c>
+      <c r="T113" s="22" t="s">
+        <v>44</v>
+      </c>
       <c r="U113" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V113" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="W113" s="21"/>
-      <c r="X113" s="21"/>
+      <c r="W113" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="X113" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="Y113" s="12"/>
     </row>
     <row r="114" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A114" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="B114" s="39" t="s">
-        <v>292</v>
+      <c r="B114" s="20" t="s">
+        <v>214</v>
       </c>
       <c r="C114" s="21"/>
       <c r="D114" s="22" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E114" s="23" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F114" s="22" t="s">
         <v>38</v>
@@ -8213,12 +8227,14 @@
         <v>39</v>
       </c>
       <c r="K114" s="22" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="L114" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M114" s="21"/>
+        <v>37</v>
+      </c>
+      <c r="M114" s="22" t="s">
+        <v>39</v>
+      </c>
       <c r="N114" s="22" t="s">
         <v>38</v>
       </c>
@@ -8228,13 +8244,15 @@
         <v>39</v>
       </c>
       <c r="R114" s="22" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="S114" s="22" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="T114" s="21"/>
-      <c r="U114" s="21"/>
+      <c r="U114" s="22" t="s">
+        <v>40</v>
+      </c>
       <c r="V114" s="22" t="s">
         <v>44</v>
       </c>
@@ -8244,10 +8262,10 @@
     </row>
     <row r="115" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A115" s="20" t="s">
-        <v>215</v>
-      </c>
-      <c r="B115" s="20" t="s">
-        <v>216</v>
+        <v>168</v>
+      </c>
+      <c r="B115" s="39" t="s">
+        <v>292</v>
       </c>
       <c r="C115" s="21"/>
       <c r="D115" s="22" t="s">
@@ -8259,17 +8277,11 @@
       <c r="F115" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="G115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="H115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="I115" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="G115" s="21"/>
+      <c r="H115" s="21"/>
+      <c r="I115" s="21"/>
       <c r="J115" s="22" t="s">
-        <v>217</v>
+        <v>39</v>
       </c>
       <c r="K115" s="22" t="s">
         <v>38</v>
@@ -8277,52 +8289,36 @@
       <c r="L115" s="23" t="s">
         <v>38</v>
       </c>
-      <c r="M115" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="M115" s="21"/>
       <c r="N115" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="O115" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P115" s="22" t="s">
-        <v>39</v>
-      </c>
+      <c r="O115" s="21"/>
+      <c r="P115" s="21"/>
       <c r="Q115" s="22" t="s">
-        <v>217</v>
+        <v>39</v>
       </c>
       <c r="R115" s="22" t="s">
-        <v>218</v>
+        <v>44</v>
       </c>
       <c r="S115" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="T115" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U115" s="22" t="s">
-        <v>39</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="T115" s="21"/>
+      <c r="U115" s="21"/>
       <c r="V115" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="W115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="X115" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y115" s="42" t="s">
-        <v>219</v>
-      </c>
+      <c r="W115" s="21"/>
+      <c r="X115" s="21"/>
+      <c r="Y115" s="12"/>
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">
         <v>215</v>
       </c>
       <c r="B116" s="20" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="22" t="s">
@@ -8388,18 +8384,20 @@
       <c r="X116" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y116" s="42"/>
+      <c r="Y116" s="42" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="20" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C117" s="21"/>
       <c r="D117" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E117" s="23" t="s">
         <v>38</v>
@@ -8417,10 +8415,10 @@
         <v>39</v>
       </c>
       <c r="J117" s="22" t="s">
-        <v>39</v>
+        <v>217</v>
       </c>
       <c r="K117" s="22" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="L117" s="23" t="s">
         <v>38</v>
@@ -8438,37 +8436,37 @@
         <v>39</v>
       </c>
       <c r="Q117" s="22" t="s">
-        <v>39</v>
+        <v>217</v>
       </c>
       <c r="R117" s="22" t="s">
-        <v>42</v>
+        <v>218</v>
       </c>
       <c r="S117" s="22" t="s">
-        <v>40</v>
+        <v>217</v>
       </c>
       <c r="T117" s="22" t="s">
         <v>44</v>
       </c>
       <c r="U117" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="V117" s="22" t="s">
         <v>44</v>
       </c>
       <c r="W117" s="22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="X117" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="Y117" s="12"/>
+        <v>39</v>
+      </c>
+      <c r="Y117" s="42"/>
     </row>
     <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="20" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="B118" s="20" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="C118" s="21"/>
       <c r="D118" s="22" t="s">
@@ -8534,77 +8532,103 @@
       <c r="X118" s="22" t="s">
         <v>40</v>
       </c>
-      <c r="Y118" s="13"/>
+      <c r="Y118" s="12"/>
     </row>
     <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="20" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="C119" s="21"/>
       <c r="D119" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E119" s="25"/>
-      <c r="F119" s="21"/>
-      <c r="G119" s="21"/>
-      <c r="H119" s="21"/>
-      <c r="I119" s="21"/>
-      <c r="J119" s="21"/>
-      <c r="K119" s="21"/>
-      <c r="L119" s="25"/>
-      <c r="M119" s="21"/>
-      <c r="N119" s="21"/>
-      <c r="O119" s="21"/>
-      <c r="P119" s="21"/>
-      <c r="Q119" s="21"/>
-      <c r="R119" s="21"/>
-      <c r="S119" s="21"/>
-      <c r="T119" s="21"/>
-      <c r="U119" s="21"/>
-      <c r="V119" s="21"/>
-      <c r="W119" s="21"/>
-      <c r="X119" s="21"/>
-      <c r="Y119" s="32" t="s">
-        <v>225</v>
-      </c>
+      <c r="E119" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F119" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="G119" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="H119" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="I119" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="J119" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="K119" s="22" t="s">
+        <v>41</v>
+      </c>
+      <c r="L119" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M119" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N119" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O119" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P119" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q119" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="R119" s="22" t="s">
+        <v>42</v>
+      </c>
+      <c r="S119" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="T119" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U119" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="V119" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="W119" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="X119" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y119" s="13"/>
     </row>
     <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B120" s="20" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C120" s="21"/>
       <c r="D120" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E120" s="25"/>
-      <c r="F120" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="G120" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="H120" s="22" t="s">
-        <v>46</v>
-      </c>
+      <c r="F120" s="21"/>
+      <c r="G120" s="21"/>
+      <c r="H120" s="21"/>
       <c r="I120" s="21"/>
       <c r="J120" s="21"/>
       <c r="K120" s="21"/>
       <c r="L120" s="25"/>
-      <c r="M120" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="N120" s="22" t="s">
-        <v>46</v>
-      </c>
-      <c r="O120" s="22" t="s">
-        <v>46</v>
-      </c>
+      <c r="M120" s="21"/>
+      <c r="N120" s="21"/>
+      <c r="O120" s="21"/>
       <c r="P120" s="21"/>
       <c r="Q120" s="21"/>
       <c r="R120" s="21"/>
@@ -8614,30 +8638,44 @@
       <c r="V120" s="21"/>
       <c r="W120" s="21"/>
       <c r="X120" s="21"/>
-      <c r="Y120" s="33"/>
+      <c r="Y120" s="32" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C121" s="21"/>
       <c r="D121" s="22" t="s">
         <v>41</v>
       </c>
       <c r="E121" s="25"/>
-      <c r="F121" s="21"/>
-      <c r="G121" s="21"/>
-      <c r="H121" s="21"/>
+      <c r="F121" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="G121" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="H121" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="I121" s="21"/>
       <c r="J121" s="21"/>
       <c r="K121" s="21"/>
       <c r="L121" s="25"/>
-      <c r="M121" s="21"/>
-      <c r="N121" s="21"/>
-      <c r="O121" s="21"/>
+      <c r="M121" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="N121" s="22" t="s">
+        <v>46</v>
+      </c>
+      <c r="O121" s="22" t="s">
+        <v>46</v>
+      </c>
       <c r="P121" s="21"/>
       <c r="Q121" s="21"/>
       <c r="R121" s="21"/>
@@ -8647,14 +8685,14 @@
       <c r="V121" s="21"/>
       <c r="W121" s="21"/>
       <c r="X121" s="21"/>
-      <c r="Y121" s="12"/>
+      <c r="Y121" s="33"/>
     </row>
     <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B122" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C122" s="21"/>
       <c r="D122" s="22" t="s">
@@ -8686,8 +8724,8 @@
       <c r="A123" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B123" s="39" t="s">
-        <v>229</v>
+      <c r="B123" s="20" t="s">
+        <v>228</v>
       </c>
       <c r="C123" s="21"/>
       <c r="D123" s="22" t="s">
@@ -8719,8 +8757,8 @@
       <c r="A124" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B124" s="20" t="s">
-        <v>230</v>
+      <c r="B124" s="39" t="s">
+        <v>229</v>
       </c>
       <c r="C124" s="21"/>
       <c r="D124" s="22" t="s">
@@ -8753,7 +8791,7 @@
         <v>223</v>
       </c>
       <c r="B125" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C125" s="21"/>
       <c r="D125" s="22" t="s">
@@ -8786,7 +8824,7 @@
         <v>223</v>
       </c>
       <c r="B126" s="20" t="s">
-        <v>83</v>
+        <v>231</v>
       </c>
       <c r="C126" s="21"/>
       <c r="D126" s="22" t="s">
@@ -8819,7 +8857,7 @@
         <v>223</v>
       </c>
       <c r="B127" s="20" t="s">
-        <v>232</v>
+        <v>83</v>
       </c>
       <c r="C127" s="21"/>
       <c r="D127" s="22" t="s">
@@ -8852,7 +8890,7 @@
         <v>223</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C128" s="21"/>
       <c r="D128" s="22" t="s">
@@ -8885,7 +8923,7 @@
         <v>223</v>
       </c>
       <c r="B129" s="20" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C129" s="21"/>
       <c r="D129" s="22" t="s">
@@ -8918,7 +8956,7 @@
         <v>223</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C130" s="21"/>
       <c r="D130" s="22" t="s">
@@ -8951,7 +8989,7 @@
         <v>223</v>
       </c>
       <c r="B131" s="20" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C131" s="21"/>
       <c r="D131" s="22" t="s">
@@ -8984,7 +9022,7 @@
         <v>223</v>
       </c>
       <c r="B132" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C132" s="21"/>
       <c r="D132" s="22" t="s">
@@ -9012,12 +9050,12 @@
       <c r="X132" s="21"/>
       <c r="Y132" s="12"/>
     </row>
-    <row r="133" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="20" t="s">
         <v>223</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C133" s="21"/>
       <c r="D133" s="22" t="s">
@@ -9050,7 +9088,7 @@
         <v>223</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C134" s="21"/>
       <c r="D134" s="22" t="s">
@@ -9083,7 +9121,7 @@
         <v>223</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C135" s="21"/>
       <c r="D135" s="22" t="s">
@@ -9116,7 +9154,7 @@
         <v>223</v>
       </c>
       <c r="B136" s="20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C136" s="21"/>
       <c r="D136" s="22" t="s">
@@ -9149,7 +9187,7 @@
         <v>223</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C137" s="21"/>
       <c r="D137" s="22" t="s">
@@ -9182,7 +9220,7 @@
         <v>223</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>76</v>
+        <v>242</v>
       </c>
       <c r="C138" s="21"/>
       <c r="D138" s="22" t="s">
@@ -9215,11 +9253,11 @@
         <v>223</v>
       </c>
       <c r="B139" s="20" t="s">
-        <v>243</v>
+        <v>76</v>
       </c>
       <c r="C139" s="21"/>
       <c r="D139" s="22" t="s">
-        <v>108</v>
+        <v>41</v>
       </c>
       <c r="E139" s="25"/>
       <c r="F139" s="21"/>
@@ -9248,11 +9286,11 @@
         <v>223</v>
       </c>
       <c r="B140" s="20" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C140" s="21"/>
       <c r="D140" s="22" t="s">
-        <v>41</v>
+        <v>108</v>
       </c>
       <c r="E140" s="25"/>
       <c r="F140" s="21"/>
@@ -9280,8 +9318,8 @@
       <c r="A141" s="20" t="s">
         <v>223</v>
       </c>
-      <c r="B141" s="39" t="s">
-        <v>280</v>
+      <c r="B141" s="20" t="s">
+        <v>244</v>
       </c>
       <c r="C141" s="21"/>
       <c r="D141" s="22" t="s">
@@ -9311,134 +9349,167 @@
     </row>
     <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="20" t="s">
-        <v>245</v>
-      </c>
-      <c r="B142" s="20" t="s">
-        <v>246</v>
-      </c>
-      <c r="C142" s="12"/>
+        <v>223</v>
+      </c>
+      <c r="B142" s="39" t="s">
+        <v>280</v>
+      </c>
+      <c r="C142" s="21"/>
       <c r="D142" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="E142" s="34"/>
-      <c r="F142" s="12"/>
-      <c r="G142" s="12"/>
-      <c r="H142" s="12"/>
-      <c r="I142" s="12"/>
-      <c r="J142" s="12"/>
-      <c r="K142" s="12"/>
-      <c r="L142" s="34"/>
-      <c r="M142" s="12"/>
-      <c r="N142" s="12"/>
-      <c r="O142" s="12"/>
-      <c r="P142" s="12"/>
-      <c r="Q142" s="12"/>
-      <c r="R142" s="12"/>
-      <c r="S142" s="12"/>
-      <c r="T142" s="12"/>
-      <c r="U142" s="12"/>
-      <c r="V142" s="12"/>
-      <c r="W142" s="12"/>
-      <c r="X142" s="12"/>
+      <c r="E142" s="25"/>
+      <c r="F142" s="21"/>
+      <c r="G142" s="21"/>
+      <c r="H142" s="21"/>
+      <c r="I142" s="21"/>
+      <c r="J142" s="21"/>
+      <c r="K142" s="21"/>
+      <c r="L142" s="25"/>
+      <c r="M142" s="21"/>
+      <c r="N142" s="21"/>
+      <c r="O142" s="21"/>
+      <c r="P142" s="21"/>
+      <c r="Q142" s="21"/>
+      <c r="R142" s="21"/>
+      <c r="S142" s="21"/>
+      <c r="T142" s="21"/>
+      <c r="U142" s="21"/>
+      <c r="V142" s="21"/>
+      <c r="W142" s="21"/>
+      <c r="X142" s="21"/>
       <c r="Y142" s="12"/>
     </row>
     <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="20" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B143" s="20" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C143" s="12"/>
       <c r="D143" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="E143" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="F143" s="21"/>
-      <c r="G143" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="H143" s="21"/>
-      <c r="I143" s="21"/>
-      <c r="J143" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="K143" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="L143" s="23" t="s">
-        <v>249</v>
-      </c>
-      <c r="M143" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="N143" s="22" t="s">
-        <v>249</v>
-      </c>
-      <c r="O143" s="21"/>
-      <c r="P143" s="21"/>
-      <c r="Q143" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="R143" s="22" t="s">
-        <v>251</v>
-      </c>
-      <c r="S143" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="T143" s="21"/>
-      <c r="U143" s="22" t="s">
-        <v>250</v>
-      </c>
-      <c r="V143" s="21"/>
-      <c r="W143" s="21"/>
-      <c r="X143" s="21"/>
+        <v>41</v>
+      </c>
+      <c r="E143" s="34"/>
+      <c r="F143" s="12"/>
+      <c r="G143" s="12"/>
+      <c r="H143" s="12"/>
+      <c r="I143" s="12"/>
+      <c r="J143" s="12"/>
+      <c r="K143" s="12"/>
+      <c r="L143" s="34"/>
+      <c r="M143" s="12"/>
+      <c r="N143" s="12"/>
+      <c r="O143" s="12"/>
+      <c r="P143" s="12"/>
+      <c r="Q143" s="12"/>
+      <c r="R143" s="12"/>
+      <c r="S143" s="12"/>
+      <c r="T143" s="12"/>
+      <c r="U143" s="12"/>
+      <c r="V143" s="12"/>
+      <c r="W143" s="12"/>
+      <c r="X143" s="12"/>
       <c r="Y143" s="12"/>
     </row>
     <row r="144" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A144" s="20" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B144" s="20" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C144" s="12"/>
       <c r="D144" s="22" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="E144" s="23" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="F144" s="21"/>
-      <c r="G144" s="21"/>
+      <c r="G144" s="22" t="s">
+        <v>249</v>
+      </c>
       <c r="H144" s="21"/>
       <c r="I144" s="21"/>
-      <c r="J144" s="21"/>
+      <c r="J144" s="22" t="s">
+        <v>250</v>
+      </c>
       <c r="K144" s="22" t="s">
-        <v>38</v>
+        <v>249</v>
       </c>
       <c r="L144" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M144" s="21"/>
-      <c r="N144" s="21"/>
+        <v>249</v>
+      </c>
+      <c r="M144" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="N144" s="22" t="s">
+        <v>249</v>
+      </c>
       <c r="O144" s="21"/>
       <c r="P144" s="21"/>
-      <c r="Q144" s="21"/>
-      <c r="R144" s="21"/>
-      <c r="S144" s="21"/>
+      <c r="Q144" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="R144" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="S144" s="22" t="s">
+        <v>250</v>
+      </c>
       <c r="T144" s="21"/>
-      <c r="U144" s="21"/>
+      <c r="U144" s="22" t="s">
+        <v>250</v>
+      </c>
       <c r="V144" s="21"/>
       <c r="W144" s="21"/>
       <c r="X144" s="21"/>
       <c r="Y144" s="12"/>
     </row>
+    <row r="145" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A145" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="B145" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="C145" s="12"/>
+      <c r="D145" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="E145" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F145" s="21"/>
+      <c r="G145" s="21"/>
+      <c r="H145" s="21"/>
+      <c r="I145" s="21"/>
+      <c r="J145" s="21"/>
+      <c r="K145" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L145" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M145" s="21"/>
+      <c r="N145" s="21"/>
+      <c r="O145" s="21"/>
+      <c r="P145" s="21"/>
+      <c r="Q145" s="21"/>
+      <c r="R145" s="21"/>
+      <c r="S145" s="21"/>
+      <c r="T145" s="21"/>
+      <c r="U145" s="21"/>
+      <c r="V145" s="21"/>
+      <c r="W145" s="21"/>
+      <c r="X145" s="21"/>
+      <c r="Y145" s="12"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="Y115:Y116"/>
+    <mergeCell ref="Y116:Y117"/>
     <mergeCell ref="C1:O1"/>
     <mergeCell ref="C2:O2"/>
     <mergeCell ref="C5:H5"/>

</xml_diff>

<commit_message>
Nimeä vanha vastaanottotarkastusraportti uusiksi, jotta uuden voi tehdä
</commit_message>
<xml_diff>
--- a/resources/roolit.xlsx
+++ b/resources/roolit.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markusva/repos/Github/harja/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57BA7F91-4BAF-F64C-8854-7A35EA535044}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21DA38DF-1251-4649-8E4D-5DFEBDE14DFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40160" yWindow="-5300" windowWidth="34560" windowHeight="21580" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -689,9 +689,6 @@
     <t>Ylläpidon aikataulu</t>
   </si>
   <si>
-    <t>Vastaanottotarkastusraportti</t>
-  </si>
-  <si>
     <t>Häiriötilanteet</t>
   </si>
   <si>
@@ -948,6 +945,9 @@
   </si>
   <si>
     <t>Vastaanottotarkastusraportti - MHU</t>
+  </si>
+  <si>
+    <t>Vastaanottotarkastusraportti - Päällystys</t>
   </si>
 </sst>
 </file>
@@ -1214,16 +1214,6 @@
     <xf numFmtId="49" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1237,6 +1227,16 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -1607,21 +1607,21 @@
       <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="43" t="s">
+      <c r="C1" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="43"/>
-      <c r="E1" s="43"/>
-      <c r="F1" s="43"/>
-      <c r="G1" s="43"/>
-      <c r="H1" s="43"/>
-      <c r="I1" s="43"/>
-      <c r="J1" s="43"/>
-      <c r="K1" s="43"/>
-      <c r="L1" s="43"/>
-      <c r="M1" s="43"/>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="J1" s="48"/>
+      <c r="K1" s="48"/>
+      <c r="L1" s="48"/>
+      <c r="M1" s="48"/>
+      <c r="N1" s="48"/>
+      <c r="O1" s="48"/>
       <c r="P1" s="2"/>
       <c r="Q1" s="2"/>
       <c r="R1" s="2"/>
@@ -1636,21 +1636,21 @@
     <row r="2" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
-      <c r="C2" s="44" t="s">
+      <c r="C2" s="49" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="44"/>
-      <c r="E2" s="44"/>
-      <c r="F2" s="44"/>
-      <c r="G2" s="44"/>
-      <c r="H2" s="44"/>
-      <c r="I2" s="44"/>
-      <c r="J2" s="44"/>
-      <c r="K2" s="44"/>
-      <c r="L2" s="44"/>
-      <c r="M2" s="44"/>
-      <c r="N2" s="44"/>
-      <c r="O2" s="44"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
+      <c r="H2" s="49"/>
+      <c r="I2" s="49"/>
+      <c r="J2" s="49"/>
+      <c r="K2" s="49"/>
+      <c r="L2" s="49"/>
+      <c r="M2" s="49"/>
+      <c r="N2" s="49"/>
+      <c r="O2" s="49"/>
       <c r="P2" s="2"/>
       <c r="Q2" s="2"/>
       <c r="R2" s="2"/>
@@ -1727,34 +1727,34 @@
     <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="12"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="45" t="s">
+      <c r="C5" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="50"/>
+      <c r="G5" s="50"/>
+      <c r="H5" s="50"/>
       <c r="I5" s="13"/>
       <c r="J5" s="13"/>
-      <c r="K5" s="45" t="s">
+      <c r="K5" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="L5" s="45"/>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
+      <c r="L5" s="50"/>
+      <c r="M5" s="50"/>
+      <c r="N5" s="50"/>
+      <c r="O5" s="50"/>
       <c r="P5" s="13"/>
       <c r="Q5" s="13"/>
-      <c r="R5" s="45" t="s">
+      <c r="R5" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="45"/>
-      <c r="V5" s="45"/>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
+      <c r="S5" s="50"/>
+      <c r="T5" s="50"/>
+      <c r="U5" s="50"/>
+      <c r="V5" s="50"/>
+      <c r="W5" s="50"/>
+      <c r="X5" s="50"/>
       <c r="Y5" s="14" t="s">
         <v>10</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>34</v>
       </c>
       <c r="B15" s="39" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="41" t="s">
@@ -2854,46 +2854,46 @@
       </c>
       <c r="C24" s="21"/>
       <c r="D24" s="22" t="s">
+        <v>287</v>
+      </c>
+      <c r="E24" s="23" t="s">
+        <v>289</v>
+      </c>
+      <c r="F24" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="E24" s="23" t="s">
+      <c r="G24" s="22" t="s">
         <v>290</v>
       </c>
-      <c r="F24" s="22" t="s">
+      <c r="H24" s="22" t="s">
+        <v>288</v>
+      </c>
+      <c r="I24" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="J24" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="K24" s="22" t="s">
+        <v>287</v>
+      </c>
+      <c r="L24" s="23" t="s">
         <v>289</v>
       </c>
-      <c r="G24" s="22" t="s">
-        <v>291</v>
-      </c>
-      <c r="H24" s="22" t="s">
-        <v>289</v>
-      </c>
-      <c r="I24" s="22" t="s">
+      <c r="M24" s="22" t="s">
         <v>286</v>
       </c>
-      <c r="J24" s="22" t="s">
-        <v>287</v>
-      </c>
-      <c r="K24" s="22" t="s">
+      <c r="N24" s="22" t="s">
         <v>288</v>
       </c>
-      <c r="L24" s="23" t="s">
-        <v>290</v>
-      </c>
-      <c r="M24" s="22" t="s">
-        <v>287</v>
-      </c>
-      <c r="N24" s="22" t="s">
-        <v>289</v>
-      </c>
       <c r="O24" s="22" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="P24" s="22" t="s">
+        <v>285</v>
+      </c>
+      <c r="Q24" s="22" t="s">
         <v>286</v>
-      </c>
-      <c r="Q24" s="22" t="s">
-        <v>287</v>
       </c>
       <c r="R24" s="22" t="s">
         <v>42</v>
@@ -3063,10 +3063,10 @@
       </c>
       <c r="C27" s="21"/>
       <c r="D27" s="41" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="F27" s="22" t="s">
         <v>38</v>
@@ -3084,10 +3084,10 @@
         <v>72</v>
       </c>
       <c r="K27" s="41" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="L27" s="40" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="M27" s="22" t="s">
         <v>39</v>
@@ -7561,8 +7561,8 @@
       <c r="A104" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="B104" s="20" t="s">
-        <v>207</v>
+      <c r="B104" s="39" t="s">
+        <v>293</v>
       </c>
       <c r="C104" s="21"/>
       <c r="D104" s="22" t="s">
@@ -7614,61 +7614,61 @@
       <c r="A105" s="39" t="s">
         <v>168</v>
       </c>
-      <c r="B105" s="46" t="s">
-        <v>293</v>
-      </c>
-      <c r="C105" s="47"/>
-      <c r="D105" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="E105" s="49" t="s">
-        <v>38</v>
-      </c>
-      <c r="F105" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="G105" s="47"/>
-      <c r="H105" s="47"/>
-      <c r="I105" s="47"/>
-      <c r="J105" s="48" t="s">
-        <v>39</v>
-      </c>
-      <c r="K105" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="L105" s="49" t="s">
-        <v>38</v>
-      </c>
-      <c r="M105" s="47"/>
-      <c r="N105" s="48" t="s">
-        <v>38</v>
-      </c>
-      <c r="O105" s="47"/>
-      <c r="P105" s="47"/>
-      <c r="Q105" s="48" t="s">
-        <v>39</v>
-      </c>
-      <c r="R105" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="S105" s="48" t="s">
-        <v>39</v>
-      </c>
-      <c r="T105" s="47"/>
-      <c r="U105" s="47"/>
-      <c r="V105" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="W105" s="47"/>
-      <c r="X105" s="47"/>
-      <c r="Y105" s="50"/>
+      <c r="B105" s="42" t="s">
+        <v>292</v>
+      </c>
+      <c r="C105" s="43"/>
+      <c r="D105" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="E105" s="45" t="s">
+        <v>38</v>
+      </c>
+      <c r="F105" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="G105" s="43"/>
+      <c r="H105" s="43"/>
+      <c r="I105" s="43"/>
+      <c r="J105" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="K105" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="L105" s="45" t="s">
+        <v>38</v>
+      </c>
+      <c r="M105" s="43"/>
+      <c r="N105" s="44" t="s">
+        <v>38</v>
+      </c>
+      <c r="O105" s="43"/>
+      <c r="P105" s="43"/>
+      <c r="Q105" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="R105" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="S105" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="T105" s="43"/>
+      <c r="U105" s="43"/>
+      <c r="V105" s="44" t="s">
+        <v>44</v>
+      </c>
+      <c r="W105" s="43"/>
+      <c r="X105" s="43"/>
+      <c r="Y105" s="46"/>
     </row>
     <row r="106" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A106" s="20" t="s">
         <v>168</v>
       </c>
       <c r="B106" s="20" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C106" s="21"/>
       <c r="D106" s="22" t="s">
@@ -7741,7 +7741,7 @@
         <v>168</v>
       </c>
       <c r="B107" s="20" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C107" s="21"/>
       <c r="D107" s="22" t="s">
@@ -7814,7 +7814,7 @@
         <v>168</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C108" s="21"/>
       <c r="D108" s="22" t="s">
@@ -7887,7 +7887,7 @@
         <v>168</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C109" s="21"/>
       <c r="D109" s="22" t="s">
@@ -7958,7 +7958,7 @@
         <v>168</v>
       </c>
       <c r="B110" s="20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C110" s="21"/>
       <c r="D110" s="22" t="s">
@@ -7991,7 +7991,7 @@
         <v>168</v>
       </c>
       <c r="B111" s="39" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C111" s="21"/>
       <c r="D111" s="22" t="s">
@@ -8062,7 +8062,7 @@
         <v>168</v>
       </c>
       <c r="B112" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C112" s="21"/>
       <c r="D112" s="22" t="s">
@@ -8208,7 +8208,7 @@
         <v>168</v>
       </c>
       <c r="B114" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C114" s="21"/>
       <c r="D114" s="22" t="s">
@@ -8265,7 +8265,7 @@
         <v>168</v>
       </c>
       <c r="B115" s="39" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C115" s="21"/>
       <c r="D115" s="22" t="s">
@@ -8315,10 +8315,10 @@
     </row>
     <row r="116" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A116" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="B116" s="20" t="s">
         <v>215</v>
-      </c>
-      <c r="B116" s="20" t="s">
-        <v>216</v>
       </c>
       <c r="C116" s="21"/>
       <c r="D116" s="22" t="s">
@@ -8340,60 +8340,60 @@
         <v>39</v>
       </c>
       <c r="J116" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="K116" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L116" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M116" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N116" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O116" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P116" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q116" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="R116" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="K116" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L116" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M116" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="N116" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O116" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P116" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q116" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="R116" s="22" t="s">
+      <c r="S116" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="T116" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="U116" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="V116" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="W116" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="X116" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y116" s="47" t="s">
         <v>218</v>
-      </c>
-      <c r="S116" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="T116" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="U116" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="V116" s="22" t="s">
-        <v>44</v>
-      </c>
-      <c r="W116" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="X116" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Y116" s="42" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="117" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A117" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B117" s="20" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C117" s="21"/>
       <c r="D117" s="22" t="s">
@@ -8415,34 +8415,34 @@
         <v>39</v>
       </c>
       <c r="J117" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="K117" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="L117" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="M117" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="N117" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="O117" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="P117" s="22" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q117" s="22" t="s">
+        <v>216</v>
+      </c>
+      <c r="R117" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="K117" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="L117" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="M117" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="N117" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="O117" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="P117" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="Q117" s="22" t="s">
-        <v>217</v>
-      </c>
-      <c r="R117" s="22" t="s">
-        <v>218</v>
-      </c>
       <c r="S117" s="22" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="T117" s="22" t="s">
         <v>44</v>
@@ -8459,14 +8459,14 @@
       <c r="X117" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="Y117" s="42"/>
+      <c r="Y117" s="47"/>
     </row>
     <row r="118" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A118" s="20" t="s">
+        <v>220</v>
+      </c>
+      <c r="B118" s="20" t="s">
         <v>221</v>
-      </c>
-      <c r="B118" s="20" t="s">
-        <v>222</v>
       </c>
       <c r="C118" s="21"/>
       <c r="D118" s="22" t="s">
@@ -8536,10 +8536,10 @@
     </row>
     <row r="119" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A119" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B119" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C119" s="21"/>
       <c r="D119" s="22" t="s">
@@ -8609,10 +8609,10 @@
     </row>
     <row r="120" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A120" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="B120" s="20" t="s">
         <v>223</v>
-      </c>
-      <c r="B120" s="20" t="s">
-        <v>224</v>
       </c>
       <c r="C120" s="21"/>
       <c r="D120" s="22" t="s">
@@ -8639,15 +8639,15 @@
       <c r="W120" s="21"/>
       <c r="X120" s="21"/>
       <c r="Y120" s="32" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="121" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A121" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B121" s="20" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C121" s="21"/>
       <c r="D121" s="22" t="s">
@@ -8689,10 +8689,10 @@
     </row>
     <row r="122" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A122" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B122" s="20" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C122" s="21"/>
       <c r="D122" s="22" t="s">
@@ -8722,10 +8722,10 @@
     </row>
     <row r="123" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A123" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B123" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C123" s="21"/>
       <c r="D123" s="22" t="s">
@@ -8755,10 +8755,10 @@
     </row>
     <row r="124" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A124" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B124" s="39" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C124" s="21"/>
       <c r="D124" s="22" t="s">
@@ -8788,10 +8788,10 @@
     </row>
     <row r="125" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A125" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B125" s="20" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C125" s="21"/>
       <c r="D125" s="22" t="s">
@@ -8821,10 +8821,10 @@
     </row>
     <row r="126" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A126" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B126" s="20" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C126" s="21"/>
       <c r="D126" s="22" t="s">
@@ -8854,7 +8854,7 @@
     </row>
     <row r="127" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A127" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B127" s="20" t="s">
         <v>83</v>
@@ -8887,10 +8887,10 @@
     </row>
     <row r="128" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A128" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B128" s="20" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C128" s="21"/>
       <c r="D128" s="22" t="s">
@@ -8920,10 +8920,10 @@
     </row>
     <row r="129" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B129" s="20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C129" s="21"/>
       <c r="D129" s="22" t="s">
@@ -8953,10 +8953,10 @@
     </row>
     <row r="130" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A130" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B130" s="20" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C130" s="21"/>
       <c r="D130" s="22" t="s">
@@ -8986,10 +8986,10 @@
     </row>
     <row r="131" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A131" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B131" s="20" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C131" s="21"/>
       <c r="D131" s="22" t="s">
@@ -9019,10 +9019,10 @@
     </row>
     <row r="132" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A132" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B132" s="20" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C132" s="21"/>
       <c r="D132" s="22" t="s">
@@ -9052,10 +9052,10 @@
     </row>
     <row r="133" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A133" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C133" s="21"/>
       <c r="D133" s="22" t="s">
@@ -9085,10 +9085,10 @@
     </row>
     <row r="134" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A134" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C134" s="21"/>
       <c r="D134" s="22" t="s">
@@ -9118,10 +9118,10 @@
     </row>
     <row r="135" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A135" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C135" s="21"/>
       <c r="D135" s="22" t="s">
@@ -9151,10 +9151,10 @@
     </row>
     <row r="136" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A136" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B136" s="20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C136" s="21"/>
       <c r="D136" s="22" t="s">
@@ -9184,10 +9184,10 @@
     </row>
     <row r="137" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A137" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C137" s="21"/>
       <c r="D137" s="22" t="s">
@@ -9217,10 +9217,10 @@
     </row>
     <row r="138" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A138" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C138" s="21"/>
       <c r="D138" s="22" t="s">
@@ -9250,7 +9250,7 @@
     </row>
     <row r="139" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A139" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B139" s="20" t="s">
         <v>76</v>
@@ -9283,10 +9283,10 @@
     </row>
     <row r="140" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A140" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B140" s="20" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C140" s="21"/>
       <c r="D140" s="22" t="s">
@@ -9316,10 +9316,10 @@
     </row>
     <row r="141" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A141" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B141" s="20" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C141" s="21"/>
       <c r="D141" s="22" t="s">
@@ -9349,10 +9349,10 @@
     </row>
     <row r="142" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A142" s="20" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B142" s="39" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C142" s="21"/>
       <c r="D142" s="22" t="s">
@@ -9382,10 +9382,10 @@
     </row>
     <row r="143" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A143" s="20" t="s">
+        <v>244</v>
+      </c>
+      <c r="B143" s="20" t="s">
         <v>245</v>
-      </c>
-      <c r="B143" s="20" t="s">
-        <v>246</v>
       </c>
       <c r="C143" s="12"/>
       <c r="D143" s="22" t="s">
@@ -9415,53 +9415,53 @@
     </row>
     <row r="144" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A144" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="B144" s="20" t="s">
         <v>247</v>
-      </c>
-      <c r="B144" s="20" t="s">
-        <v>248</v>
       </c>
       <c r="C144" s="12"/>
       <c r="D144" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="E144" s="23" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="F144" s="21"/>
       <c r="G144" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H144" s="21"/>
       <c r="I144" s="21"/>
       <c r="J144" s="22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="K144" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="L144" s="23" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="M144" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="N144" s="22" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="O144" s="21"/>
       <c r="P144" s="21"/>
       <c r="Q144" s="22" t="s">
+        <v>249</v>
+      </c>
+      <c r="R144" s="22" t="s">
         <v>250</v>
       </c>
-      <c r="R144" s="22" t="s">
-        <v>251</v>
-      </c>
       <c r="S144" s="22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="T144" s="21"/>
       <c r="U144" s="22" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="V144" s="21"/>
       <c r="W144" s="21"/>
@@ -9470,10 +9470,10 @@
     </row>
     <row r="145" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A145" s="20" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B145" s="20" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C145" s="12"/>
       <c r="D145" s="22" t="s">
@@ -9538,24 +9538,24 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="35" t="s">
+        <v>252</v>
+      </c>
+      <c r="B1" s="35" t="s">
         <v>253</v>
       </c>
-      <c r="B1" s="35" t="s">
+      <c r="C1" s="35" t="s">
         <v>254</v>
       </c>
-      <c r="C1" s="35" t="s">
+      <c r="D1" s="35" t="s">
         <v>255</v>
       </c>
-      <c r="D1" s="35" t="s">
+      <c r="E1" s="35" t="s">
         <v>256</v>
-      </c>
-      <c r="E1" s="35" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="36" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B2" s="36" t="s">
         <v>13</v>
@@ -9568,7 +9568,7 @@
     </row>
     <row r="3" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="36" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="B3" s="36" t="s">
         <v>15</v>
@@ -9581,7 +9581,7 @@
     </row>
     <row r="4" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="36" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="B4" s="36" t="s">
         <v>17</v>
@@ -9594,7 +9594,7 @@
     </row>
     <row r="5" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="B5" s="36" t="s">
         <v>14</v>
@@ -9603,13 +9603,13 @@
         <v>4</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E5" s="37"/>
     </row>
     <row r="6" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="36" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="B6" s="36" t="s">
         <v>16</v>
@@ -9618,13 +9618,13 @@
         <v>4</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E6" s="37"/>
     </row>
     <row r="7" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B7" s="36" t="s">
         <v>18</v>
@@ -9633,13 +9633,13 @@
         <v>4</v>
       </c>
       <c r="D7" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E7" s="37"/>
     </row>
     <row r="8" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="36" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B8" s="36" t="s">
         <v>19</v>
@@ -9648,13 +9648,13 @@
         <v>4</v>
       </c>
       <c r="D8" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E8" s="37"/>
     </row>
     <row r="9" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="36" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B9" s="36" t="s">
         <v>27</v>
@@ -9663,13 +9663,13 @@
         <v>5</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E9" s="37"/>
     </row>
     <row r="10" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="36" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B10" s="36" t="s">
         <v>20</v>
@@ -9682,7 +9682,7 @@
     </row>
     <row r="11" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="36" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B11" s="36" t="s">
         <v>23</v>
@@ -9695,7 +9695,7 @@
     </row>
     <row r="12" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="36" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B12" s="36" t="s">
         <v>24</v>
@@ -9708,7 +9708,7 @@
     </row>
     <row r="13" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B13" s="36" t="s">
         <v>21</v>
@@ -9717,13 +9717,13 @@
         <v>6</v>
       </c>
       <c r="D13" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E13" s="37"/>
     </row>
     <row r="14" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="36" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="B14" s="36" t="s">
         <v>22</v>
@@ -9732,13 +9732,13 @@
         <v>6</v>
       </c>
       <c r="D14" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E14" s="37"/>
     </row>
     <row r="15" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="36" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="B15" s="36" t="s">
         <v>25</v>
@@ -9747,13 +9747,13 @@
         <v>6</v>
       </c>
       <c r="D15" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E15" s="37"/>
     </row>
     <row r="16" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="36" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B16" s="36" t="s">
         <v>26</v>
@@ -9762,13 +9762,13 @@
         <v>6</v>
       </c>
       <c r="D16" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E16" s="37"/>
     </row>
     <row r="17" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="36" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B17" s="36" t="s">
         <v>29</v>
@@ -9777,13 +9777,13 @@
         <v>5</v>
       </c>
       <c r="D17" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E17" s="37"/>
     </row>
     <row r="18" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="36" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B18" s="36" t="s">
         <v>31</v>
@@ -9792,13 +9792,13 @@
         <v>5</v>
       </c>
       <c r="D18" s="38" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="E18" s="37"/>
     </row>
     <row r="19" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="36" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="B19" s="36" t="s">
         <v>28</v>
@@ -9807,13 +9807,13 @@
         <v>5</v>
       </c>
       <c r="D19" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E19" s="37"/>
     </row>
     <row r="20" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="36" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="B20" s="36" t="s">
         <v>30</v>
@@ -9822,7 +9822,7 @@
         <v>5</v>
       </c>
       <c r="D20" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E20" s="37"/>
     </row>
@@ -9837,13 +9837,13 @@
         <v>5</v>
       </c>
       <c r="D21" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E21" s="37"/>
     </row>
     <row r="22" spans="1:5" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="36" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B22" s="36" t="s">
         <v>32</v>
@@ -9852,7 +9852,7 @@
         <v>5</v>
       </c>
       <c r="D22" s="38" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="E22" s="37"/>
     </row>

</xml_diff>